<commit_message>
SCRUM-39: Execute Test Case Employee/Manager
</commit_message>
<xml_diff>
--- a/Docs/Test-Case/Test_Case_Authorization.xlsx
+++ b/Docs/Test-Case/Test_Case_Authorization.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1497,6 +1497,313 @@
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>BOUNDARY VALUE ANALYSIS (BVA) - API LEVEL</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_01</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra đăng ký với Password có độ dài 2 ký tự (giá trị dưới biên)</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>API /register hoạt động; Email chưa tồn tại.</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /register.
+2. Nhập Password: 12.
+3. Nhập các thông tin User hợp lệ khác.
+4. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request do Password phải có tối thiểu 3 ký tự.</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>NG – API trả 200 OK</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>BUG-BVA-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_02</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra đăng ký với Password = 3 ký tự</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>API đăng ký hoạt động, email chưa tồn tại.</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /register.
+2. Nhập Password: 123.
+3. Nhập các thông tin User hợp lệ khác.
+4. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_03</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra thêm sản phẩm vào giỏ hàng với Quantity = 0</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập Customer hợp lệ, sản phẩm tồn tại.</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /cart/add.
+2. Nhập body : {"productId": "B0001", "quantity": 0}
+3. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request do Quantity phải ≥ 1.</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>NG – API trả 200 OK, 
+body true</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>BUG-BVA-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_04</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra thêm sản phẩm vào giỏ hàng với Quantity = 1</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập Customer hợp lệ, sản phẩm tồn tại.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /cart/add.
+2. Nhập body : {"productId": "B0001", "quantity": 1}
+3. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, thêm sản phẩm thành công.</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OK </t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_05</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra tạo sản phẩm với Product Stock = -1</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập tài khoản (Manager) có quyền tạo sản phẩm.</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /seller/product/new
+2. Nhập body : 
+{
+  "productId": "B000128",
+  "productName": "Angular in Action",
+  "productPrice": 40.00,
+  "productStock": -1,
+  "productDescription": "Book for learning Angular",
+  "productIcon": "https://via.placeholder.com/150",
+  "categoryType": 0,
+  "productStatus": 0
+}
+3. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request do Product Stock phải ≥ 0.</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>NG – API trả 500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>BUG-BVA-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_06</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra tạo sản phẩm với Product Stock = 0</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập tài khoản (Manager) có quyền tạo sản phẩm.</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /seller/product/new
+2. Nhập body : 
+{
+  "productId": "B000128",
+  "productName": "Angular in Action",
+  "productPrice": 40.00,
+  "productStock": 1,
+  "productDescription": "Book for learning Angular",
+  "productIcon": "https://via.placeholder.com/150",
+  "categoryType": 0,
+  "productStatus": 0
+}
+3. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, tạo sản phẩm thành công.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>TC_API_BVA_07</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra tạo sản phẩm với Product Price = -1</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập tài khoản (Manager) có quyền tạo sản phẩm.</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi request POST /seller/product/new
+2. Nhập body : 
+{
+  "productId": "B000128",
+  "productName": "Angular in Action",
+  "productPrice": -40.00,
+  "productStock": 50,
+  "productDescription": "Book for learning Angular",
+  "productIcon": "https://via.placeholder.com/150",
+  "categoryType": 0,
+  "productStatus": 0
+}
+3. Gửi request.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request do giá sản phẩm không được âm.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>NG – API trả 200 OK</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>BUG-BVA-04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>